<commit_message>
Formato de solicitud: ortografía, numeración y aviso de obligatorios
Acentos (Mercancía, Marítimo, Aéreo, Talón, Guía, Línea aérea), la sección 2
decía "1. BENEFICIAROO", espacios en 5., 8. y 9., y el aviso inicial ahora
dice que las celdas en rojo son obligatorias y pide una solicitud por
archivo (ya se aceptan varios archivos en un correo). Solo cambian esos
textos: estilos, logo, celdas combinadas y alertas quedan iguales
(template_integrity_check pasa).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/solicitud_aseguramiento_formato_jr_preparado.xlsx
+++ b/docs/solicitud_aseguramiento_formato_jr_preparado.xlsx
@@ -20,16 +20,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="83">
   <si>
-    <t>SOLICITUD DE ASEGURAMIENTO DE MERCANCIA</t>
-  </si>
-  <si>
-    <t>Completa únicamente las celdas en Azul claro. Envie este archivo Excel como adjunto, una solicitud por correo.</t>
+    <t>SOLICITUD DE ASEGURAMIENTO DE MERCANCÍA</t>
+  </si>
+  <si>
+    <t>Llena las celdas en azul claro; las marcadas en rojo son obligatorias. Envía una solicitud por archivo Excel.</t>
   </si>
   <si>
     <t>1. SOLICITANTE</t>
   </si>
   <si>
-    <t xml:space="preserve">Solicitante </t>
+    <t>Solicitante</t>
   </si>
   <si>
     <t>Teléfono</t>
@@ -38,7 +38,7 @@
     <t>Fecha</t>
   </si>
   <si>
-    <t>1. BENEFICIAROO DEL SEGURO</t>
+    <t>2. BENEFICIARIO DEL SEGURO</t>
   </si>
   <si>
     <t>Nombre</t>
@@ -50,7 +50,7 @@
     <t>Contacto</t>
   </si>
   <si>
-    <t>3. MERCANCIA POR ASEGURAR</t>
+    <t>3. MERCANCÍA POR ASEGURAR</t>
   </si>
   <si>
     <t>Mercancía asegurada</t>
@@ -83,7 +83,7 @@
     <t>País destino</t>
   </si>
   <si>
-    <t>5.CONCEPTOS POR ASEGURAR</t>
+    <t>5. CONCEPTOS POR ASEGURAR</t>
   </si>
   <si>
     <t>Moneda</t>
@@ -110,25 +110,25 @@
     <t>7. DATOS DEL PROVEEDOR</t>
   </si>
   <si>
-    <t>8.REFERENCIAS</t>
+    <t>8. REFERENCIAS</t>
   </si>
   <si>
     <t>Terrestre</t>
   </si>
   <si>
-    <t>Maritimo</t>
-  </si>
-  <si>
-    <t>Aereo</t>
-  </si>
-  <si>
-    <t>Talon embarque</t>
+    <t>Marítimo</t>
+  </si>
+  <si>
+    <t>Aéreo</t>
+  </si>
+  <si>
+    <t>Talón embarque</t>
   </si>
   <si>
     <t>B/L</t>
   </si>
   <si>
-    <t>N° Guia</t>
+    <t>N° Guía</t>
   </si>
   <si>
     <t>N° Contenedor o caja</t>
@@ -137,13 +137,13 @@
     <t>Contenedor</t>
   </si>
   <si>
-    <t>Linea aerea</t>
-  </si>
-  <si>
-    <t>9.DECLARACIÓN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acepto que la información declarada es verídica </t>
+    <t>Línea aérea</t>
+  </si>
+  <si>
+    <t>9. DECLARACIÓN</t>
+  </si>
+  <si>
+    <t>Acepto que la información declarada es verídica</t>
   </si>
   <si>
     <r>
@@ -2365,19 +2365,19 @@
     <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Opción inválida" error="Selecciona una opción de la lista." sqref="I23">
       <formula1>"Terrestre,Marítimo,Aéreo,Multimodal"</formula1>
     </dataValidation>
-    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Capture un monto numérico." sqref="D30">
+    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Captura un monto numérico." sqref="D30">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Capture un monto numérico." sqref="I30">
+    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Captura un monto numérico." sqref="I30">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Capture un monto numérico." sqref="D31">
+    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Captura un monto numérico." sqref="D31">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Capture un monto numérico." sqref="I31">
+    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Captura un monto numérico." sqref="I31">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Capture un monto numérico." sqref="D32">
+    <dataValidation type="decimal" errorStyle="stop" operator="greaterThanOrEqual" allowBlank="0" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Captura un monto numérico." sqref="D32">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="date" errorStyle="stop" operator="between" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Escribe una fecha real, por ejemplo 24/09/2026. Si tu Excel no la acepta así, escríbela con el formato de fecha de tu computadora." promptTitle="Fecha" prompt="Escribe la fecha, por ejemplo 24/09/2026." sqref="J8:K8">

</xml_diff>

<commit_message>
Moneda obligatoria y constancia con fecha, montos y pie corregidos
- Moneda obligatoria (ValidationService::REQUIRED, que ahora usan también
  el generador del PDF y el chequeo del Excel) y solo USD o PESOS. Excel:
  alerta roja en D29; PDF: ya la marcaba.
- Pie del Excel: www.jgmylard.com (decía .com.mx, que no responde).
- Constancia (update 11009): fecha 25/09/2026 y suma "$165,000.00 USD/MXN";
  el PDF de fondo decía "JY MYLARD", "Num." y le faltaba "Valentín". Se
  corrigió reescribiendo solo esos dos renglones con sus fuentes originales
  (Century Gothic Bold, Lucida Sans Unicode); el resto del texto es idéntico.
  El update solo reemplaza el archivo si es exactamente el revisado (hash) y
  guarda el anterior como Constancia-anterior-20260928.pdf.
- template_integrity_check compara las alertas con la lista de obligatorios
  y revisa el pie; batch_reply_check prueba la moneda vacía.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/solicitud_aseguramiento_formato_jr_preparado.xlsx
+++ b/docs/solicitud_aseguramiento_formato_jr_preparado.xlsx
@@ -171,7 +171,7 @@
       <t xml:space="preserve">
 Calle 29 Núm. 69 Col. Valentín Gómez Farías C.P. 15010, Venustiano Carranza, Ciudad de México, México
 Tel. Of. +52 (55) 8943-1208, +52 (55) 8943-6064
-www.jgmylard.com.mx</t>
+www.jgmylard.com</t>
     </r>
   </si>
   <si>
@@ -785,7 +785,16 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFBD5D5"/>
+          <bgColor rgb="FFFBD5D5"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2352,6 +2361,11 @@
       <formula>LEN(TRIM($D$32))=0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D29">
+    <cfRule type="expression" dxfId="9" priority="8">
+      <formula>LEN(TRIM($D$29))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="11">
     <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="0" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="Opción inválida" error="Selecciona una opción de la lista." sqref="D19">
       <formula1>"Nueva,Usada"</formula1>

</xml_diff>